<commit_message>
feat(ai): add comprehensive Chinese translations for all 771 purged words in stage 2
</commit_message>
<xml_diff>
--- a/data/derived_outputs/stage_gold_2000/purged_new_candidates_2000.xlsx
+++ b/data/derived_outputs/stage_gold_2000/purged_new_candidates_2000.xlsx
@@ -2344,2317 +2344,2317 @@
     <t>youngest</t>
   </si>
   <si>
-    <t>normal (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>observe (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>opened (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>optimum (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pattern (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>privilege (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rewarded (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>security (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sensitivity (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>soak (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>somewhere (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tight (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unlike (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>whim (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>adjusted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>approached (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>blew (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>clearer (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>clouded (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>contrasting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>created (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>desert (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>die (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dog (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>entirely (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>expanse (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>extended (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>falling (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>finished (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>friendlier (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>giant (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>grasp (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>handful (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hence (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hood (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>immaculate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>improvement (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>jump (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>laughing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lied (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>loading (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lore (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lush (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>memorial (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>mild (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>needless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>notable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>nurse (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>older (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>proved (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>realizing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>reputation (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>responded (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>riley (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rocky (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shade (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shame (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sheep (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shut (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>spite (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>struck (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>thrown (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>treasure (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>treatment (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>wondering (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>accepted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>accident (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>action (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>affected (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ambassador (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>arduous (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>asleep (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>banter (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>benefited (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bored (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>boring (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>breaking (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>captured (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>careful (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>carry (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>cautious (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>clearest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>clinging (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>colorful (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>commended (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>commute (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>compliment (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>controlled (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>correspondence (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>costly (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>covering (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>crazy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>creating (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>critic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>cute (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>damn (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>daring (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>delivers (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>descending (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>deserved (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>distract (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dress (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>educating (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>enable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>enabled (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>equal (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>estimate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>everyday (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>excellence (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>exception (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>excess (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>exotic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>extending (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>extinct (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fancy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fitting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>flipped (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fragrant (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fret (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fuller (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fullest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>getaway (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>grace (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>granted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>happening (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>harbour (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hesitating (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>honesty (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hugged (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>humility (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>imperial (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>improving (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>inadequate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>incomprehensible (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>independent (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>indulge (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>injured (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>instant (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>jam (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>kindly (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lay (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>leading (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>leery (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lock (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lookout (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>luscious (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>match (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>mighty (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>mindful (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>news (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>obscured (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>optimal (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>orderly (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>penalty (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pertinent (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pinnacle (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>plain (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>practiced (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>praise (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>precision (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>puffy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pull (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ranked (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>reality (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>region (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>remaining (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>report (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rosemary (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ruining (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rush (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rust (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>school (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>secret (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>securely (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sensing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>severe (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shining (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shortest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>silly (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>slim (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>snap (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>snapped (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sometime (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>squeezed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>stability (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>staring (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>stick (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>stormy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>subject (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>subtle (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>supporting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>surface (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tale (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>talented (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tentative (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>territory (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>trained (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tropical (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>undecided (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>uneven (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unexplainable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unimaginable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unlikely (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>untouched (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>varied (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>warn (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>wasting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>abandoned (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>abrupt (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ache (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>actively (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>adamant (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>adept (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>adequate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>adjustment (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>admirably (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>admission (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>adorable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>adored (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>affect (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>aggravate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>aid (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>airy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>alike (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>alive (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>altered (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>altering (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>altogether (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>amelia (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>anticipate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>antsy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>apocalypse (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>apology (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>apparent (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>appease (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>appointed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>appreciative (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>arctic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>art (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>asset (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>assume (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>assuring (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>atrocious (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>attack (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>attesting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>attractive (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>avid (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>avoided (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>avoiding (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>award (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>babbling (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>backed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>backing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>banner (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bearable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>beating (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>beg (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>belonging (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>blanket (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>blasted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>blessing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>blindfolded (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>blip (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>blob (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>blow (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bluff (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>boiled (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bolder (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bond (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bottomless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bound (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>brain (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>brave (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>breezy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>brilliantly (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>brown (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>browse (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bug (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bumpier (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bumping (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>buoyant (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>burn (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>burned (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>burnt (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bust (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>buying (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>buzz (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>bypass (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>cast (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>catty (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>centerpiece (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>certified (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>challenge (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>champ (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>chaotic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>character (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>chargeable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>cheapest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>chicken (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>chief (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>chilled (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>cleanest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>cleanliness (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>clearing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>climbed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>closest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>cohesive (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>combine (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>combining (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>commercialized (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>committed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>compensate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>compensated (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>complained (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>completing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>complex (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>compliance (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>complimented (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>concerning (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>confused (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>congestion (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>congratulation (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>conscience (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>considerate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>console (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>consoling (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>constructive (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>continent (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>continuous (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>contrary (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>contributed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>converted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>coordinate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>coordination (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>cornucopia (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>corresponding (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>countless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>coy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>crane (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>crappy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>crazed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>creates (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>criticism (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>crooked (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>crunch (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>crusty (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>cry (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>curt (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>damage (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dash (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>deeper (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>degraded (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>delivering (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>deluxe (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>demonstrated (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>denied (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>denying (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>desirable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>desire (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>desired (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dicey (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dickey (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>digest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>diluted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>diminish (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>disadvantage (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>disappear (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>disguise (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dislike (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dismay (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dissipate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>distortion (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>district (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>disturbing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dos (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>downfall (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>downgraded (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dramatically (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dreaming (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dressed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dubbed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dud (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>duke (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dumb (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>dynamic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>echo (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>eden (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>educate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>element (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>elusive (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>enables (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>enabling (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>encompassing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>encouragement (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>endeavor (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>endless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>endorse (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>endure (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>enhance (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>enlightening (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ethical (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>everlasting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>excellently (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>excuse (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>exhausting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>existent (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>exposure (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>extends (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>extolled (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fab (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>facing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fail (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>failing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>faint (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>false (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>familiarity (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fantasy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fat (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fatality (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>faulty (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>favor (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>favorable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>feared (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>feat (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>featured (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>feed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>final (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fired (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>firm (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>flash (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>flood (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>flooded (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>flop (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>focussed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fond (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ford (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>foremost (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>forgetting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>forgo (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>formal (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>formidable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>forthright (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>frankly (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>freak (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>freaked (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>freaking (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>friendliest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>frowning (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>fulfillment (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>funky (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>gained (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>gca (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>generic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>gimmick (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>glaciated (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>gloom (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>glow (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>goodness (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>gourmet (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>graphic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>greener (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>grip (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>gripe (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>grouping (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>gruffness (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>guaranteeing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>gushing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hairless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ham (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>handicap (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>handicraft (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hardest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>harried (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>health (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>heap (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>heating (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>heavier (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>heaviest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>heavily (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hero (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hesitancy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hint (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hitting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hole (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>homey (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>horribly (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>humble (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>humoured (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>husky (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>hygiene (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>illustrate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>inclined (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>incomparable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>independently (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>induced (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>indulged (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>industrial (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>inquired (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>inspire (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>inspires (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>instructing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>interfering (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>intolerable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>invasive (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>itching (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>jackpot (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>jarring (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>jerky (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>joked (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>kill (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>kindest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>knock (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>kudos (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>labeled (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lapse (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>largest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lean (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lecture (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>legitimacy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>leisured (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lends (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lenient (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>leper (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>limitation (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>limitless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lined (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lively (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>locking (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>loose (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lose (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>loss (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lover (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>lowered (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>magnificently (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>mar (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>marriage (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>master (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>material (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>meaningful (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>measure (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>melted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>merry (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>mess (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>method (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>minimising (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>minimizing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>minus (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>miracle (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>mitigate (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>modernized (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>modified (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>motorway (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>mule (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>musical (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>mystical (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>neck (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>nerd (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>nestled (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>nimble (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>nonetheless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>nose (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>nostalgic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>noted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>obliged (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>obnoxious (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>occur (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>occurred (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>oddly (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>outright (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>oversized (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>paraplegic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>passable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>passport (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>perception (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>perfection (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pierce (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pit (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>plastic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>playful (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pleasantness (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>poetic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>polish (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pound (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>practical (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>practice (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>precisely (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>preference (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pregnant (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>premium (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>presence (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>preserve (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pricier (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>prime (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>probability (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>prominent (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>propensity (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>prospect (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>purple (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>push (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>pushed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>questioned (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rail (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>raising (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rally (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ranking (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rapid (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>raw (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>readily (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>realised (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>recall (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>receives (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>receiving (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>recovery (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>reflecting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>reflects (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>refusing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>regent (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>relative (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>remark (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>removed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>removing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rendering (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>replaced (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>reported (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>reporting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>represent (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>represents (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rescue (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>resounding (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>responsibility (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>restraint (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>retiring (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>revived (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>revolting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>reward (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>richer (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rig (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rigorous (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rising (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>risking (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>risky (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>roaring (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rose (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>royal (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rued (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ruffling (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>ruin (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>rusty (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sacred (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sainthood (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>salt (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>salvaging (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>satisfaction (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>satisfactorily (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>satisfactory (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>seal (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sealed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>seemless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>separated (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>serve (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sexy (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shadow (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shifted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shiny (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shipwreck (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>shoot (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>signature (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sincere (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sits (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>smarter (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>smelled (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>smelling (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>snafu (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>snowed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>soften (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>soil (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>specialized (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>spoiling (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sport (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>spouting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>statement (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>steam (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>steep (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sticking (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>stiller (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>stillness (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sting (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>stinky (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>straightforward (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>stranger (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>strength (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>strenuous (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>stronger (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>substitute (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>success (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>suck (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>suffers (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sufficient (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>suited (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sunshine (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>surprising (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>suspected (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>swallow (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>swamp (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>swan (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>swear (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sweeter (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sweetheart (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>swell (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>swinging (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>sympathetic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tactile (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>taller (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>teach (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>teary (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tendency (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tender (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tends (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>test (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>thickest (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>thirsty (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>throwing (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>timeless (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>topper (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>topping (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>totality (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tragic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>transparency (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>trek (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>trick (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>tropic (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>uncharted (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>understated (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unethical (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unhelpful (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unimpressed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>uninhabited (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>uninterested (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unloaded (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unlucky (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unpaved (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unrivalled (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unsurpassable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>unusual (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>upbeat (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>vain (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>valued (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>vanish (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>vary (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>varying (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>verify (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>vernal (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>versed (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>viable (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>victory (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>waived (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>wander (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>wandered (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>warmer (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>watchful (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>weary (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>weathered (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>weep (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>wisdom (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>woke (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>yearly (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>yelling (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>yielded (中性/客观/过程/实体词)</t>
-  </si>
-  <si>
-    <t>youngest (中性/客观/过程/实体词)</t>
+    <t>normal (名词/实体)</t>
+  </si>
+  <si>
+    <t>observe (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>opened (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>optimum (名词/实体)</t>
+  </si>
+  <si>
+    <t>pattern (名词/实体)</t>
+  </si>
+  <si>
+    <t>privilege (名词/实体)</t>
+  </si>
+  <si>
+    <t>rewarded (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>security (名词/实体)</t>
+  </si>
+  <si>
+    <t>sensitivity (名词/实体)</t>
+  </si>
+  <si>
+    <t>soak (名词/实体)</t>
+  </si>
+  <si>
+    <t>somewhere (名词/实体)</t>
+  </si>
+  <si>
+    <t>tight (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unlike (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>whim (名词/实体)</t>
+  </si>
+  <si>
+    <t>adjusted (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>approached (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>blew (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>clearer (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>clouded (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>contrasting (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>created (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>desert (名词/实体)</t>
+  </si>
+  <si>
+    <t>die (名词/实体)</t>
+  </si>
+  <si>
+    <t>dog (名词/实体)</t>
+  </si>
+  <si>
+    <t>entirely (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>广袤空间 / 辽阔地带</t>
+  </si>
+  <si>
+    <t>延长的 / 扩展的</t>
+  </si>
+  <si>
+    <t>下落的 / 降落中</t>
+  </si>
+  <si>
+    <t>完成的 / 结束的</t>
+  </si>
+  <si>
+    <t>更友好的</t>
+  </si>
+  <si>
+    <t>巨大的 / 巨型的</t>
+  </si>
+  <si>
+    <t>领悟 / 掌握</t>
+  </si>
+  <si>
+    <t>少数 / 少量</t>
+  </si>
+  <si>
+    <t>因此 / 由此</t>
+  </si>
+  <si>
+    <t>机罩 / 舱盖</t>
+  </si>
+  <si>
+    <t>洁净如新的 / 完美的</t>
+  </si>
+  <si>
+    <t>改进 / 提升</t>
+  </si>
+  <si>
+    <t>跳跃 / 骤升</t>
+  </si>
+  <si>
+    <t>大笑 / 欢笑</t>
+  </si>
+  <si>
+    <t>位于 / 躺着</t>
+  </si>
+  <si>
+    <t>登机中 / 装载中</t>
+  </si>
+  <si>
+    <t>传说 / 历史掌故</t>
+  </si>
+  <si>
+    <t>郁郁葱葱的</t>
+  </si>
+  <si>
+    <t>纪念馆 / 纪念碑</t>
+  </si>
+  <si>
+    <t>温和的 / 轻微的</t>
+  </si>
+  <si>
+    <t>没必要的</t>
+  </si>
+  <si>
+    <t>显著的 / 值得注意的</t>
+  </si>
+  <si>
+    <t>照顾 / 护士</t>
+  </si>
+  <si>
+    <t>较年长的</t>
+  </si>
+  <si>
+    <t>证明是 / 证实</t>
+  </si>
+  <si>
+    <t>意识到 / 觉察到</t>
+  </si>
+  <si>
+    <t>声誉 / 名声</t>
+  </si>
+  <si>
+    <t>回应 / 答复</t>
+  </si>
+  <si>
+    <t>人名（飞行员/游客）</t>
+  </si>
+  <si>
+    <t>岩石崎岖的</t>
+  </si>
+  <si>
+    <t>遮阳 / 阴凉处</t>
+  </si>
+  <si>
+    <t>遗憾 / 可惜</t>
+  </si>
+  <si>
+    <t>野生羊 / 绵羊</t>
+  </si>
+  <si>
+    <t>关闭 / 闭合</t>
+  </si>
+  <si>
+    <t>尽管 / 恶作剧</t>
+  </si>
+  <si>
+    <t>留有深刻印象 / 碰撞</t>
+  </si>
+  <si>
+    <t>扔出 / 投掷</t>
+  </si>
+  <si>
+    <t>珍宝 / 财富</t>
+  </si>
+  <si>
+    <t>对待方式 / 款待</t>
+  </si>
+  <si>
+    <t>纳闷 / 好奇</t>
+  </si>
+  <si>
+    <t>接受的 / 认可的</t>
+  </si>
+  <si>
+    <t>意外 / 事故</t>
+  </si>
+  <si>
+    <t>动作 / 行动</t>
+  </si>
+  <si>
+    <t>受影响的</t>
+  </si>
+  <si>
+    <t>大使 / 形象代表</t>
+  </si>
+  <si>
+    <t>艰难辛苦的</t>
+  </si>
+  <si>
+    <t>睡着的</t>
+  </si>
+  <si>
+    <t>调侃 / 幽默交谈</t>
+  </si>
+  <si>
+    <t>受益 / 获益</t>
+  </si>
+  <si>
+    <t>感到无聊的</t>
+  </si>
+  <si>
+    <t>枯燥无聊的</t>
+  </si>
+  <si>
+    <t>打破 / 破碎</t>
+  </si>
+  <si>
+    <t>捕捉到 / 拍下</t>
+  </si>
+  <si>
+    <t>细心的 / 谨慎的</t>
+  </si>
+  <si>
+    <t>携带 / 运载</t>
+  </si>
+  <si>
+    <t>谨慎小心的</t>
+  </si>
+  <si>
+    <t>最清晰的</t>
+  </si>
+  <si>
+    <t>紧贴的 / 依附的</t>
+  </si>
+  <si>
+    <t>色彩斑斓的</t>
+  </si>
+  <si>
+    <t>表彰 / 称赞</t>
+  </si>
+  <si>
+    <t>往返 / 通勤</t>
+  </si>
+  <si>
+    <t>赞美 / 称赞</t>
+  </si>
+  <si>
+    <t>操控好的 / 控温的</t>
+  </si>
+  <si>
+    <t>通讯 / 信件</t>
+  </si>
+  <si>
+    <t>昂贵的 / 成本高的</t>
+  </si>
+  <si>
+    <t>覆盖 / 包含</t>
+  </si>
+  <si>
+    <t>疯狂的 / 极度的</t>
+  </si>
+  <si>
+    <t>创造 / 产生</t>
+  </si>
+  <si>
+    <t>评论家 / 批评者</t>
+  </si>
+  <si>
+    <t>可爱的</t>
+  </si>
+  <si>
+    <t>极其 / 确实（语气助词）</t>
+  </si>
+  <si>
+    <t>大胆激进的</t>
+  </si>
+  <si>
+    <t>履约 / 提供</t>
+  </si>
+  <si>
+    <t>下降俯冲的</t>
+  </si>
+  <si>
+    <t>应得的 / 理所应当</t>
+  </si>
+  <si>
+    <t>分散注意力 / 分心</t>
+  </si>
+  <si>
+    <t>着装 / 穿衣</t>
+  </si>
+  <si>
+    <t>讲解中 / 教育</t>
+  </si>
+  <si>
+    <t>使能够 / 实现</t>
+  </si>
+  <si>
+    <t>实现了 / 赋能</t>
+  </si>
+  <si>
+    <t>平等的 / 相等的</t>
+  </si>
+  <si>
+    <t>预估 / 估计</t>
+  </si>
+  <si>
+    <t>日常的 / 平日的</t>
+  </si>
+  <si>
+    <t>卓越 / 出色</t>
+  </si>
+  <si>
+    <t>例外情况</t>
+  </si>
+  <si>
+    <t>额外 / 多余的</t>
+  </si>
+  <si>
+    <t>异域风情的</t>
+  </si>
+  <si>
+    <t>延伸中 / 扩展</t>
+  </si>
+  <si>
+    <t>灭绝的 / 死火山</t>
+  </si>
+  <si>
+    <t>高档的 / 华丽的</t>
+  </si>
+  <si>
+    <t>适合的 / 恰当的</t>
+  </si>
+  <si>
+    <t>翻转 / 倒置</t>
+  </si>
+  <si>
+    <t>芳香的</t>
+  </si>
+  <si>
+    <t>挂心 / 烦恼</t>
+  </si>
+  <si>
+    <t>更充分的</t>
+  </si>
+  <si>
+    <t>最充分的</t>
+  </si>
+  <si>
+    <t>短途度假</t>
+  </si>
+  <si>
+    <t>优雅 / 风度</t>
+  </si>
+  <si>
+    <t>顺理成章 / 给予</t>
+  </si>
+  <si>
+    <t>发生中</t>
+  </si>
+  <si>
+    <t>港湾 / 海港</t>
+  </si>
+  <si>
+    <t>犹豫中</t>
+  </si>
+  <si>
+    <t>真诚 / 诚实</t>
+  </si>
+  <si>
+    <t>拥抱 / 贴近</t>
+  </si>
+  <si>
+    <t>谦逊 / 谦卑</t>
+  </si>
+  <si>
+    <t>帝王级的 / 宏大的</t>
+  </si>
+  <si>
+    <t>改善提升中</t>
+  </si>
+  <si>
+    <t>不够的 / 不足的</t>
+  </si>
+  <si>
+    <t>难以理解的</t>
+  </si>
+  <si>
+    <t>独立的</t>
+  </si>
+  <si>
+    <t>犒劳自己 / 沉溺</t>
+  </si>
+  <si>
+    <t>受伤的</t>
+  </si>
+  <si>
+    <t>即刻的 / 瞬间的</t>
+  </si>
+  <si>
+    <t>拥堵 / 阻塞</t>
+  </si>
+  <si>
+    <t>友善地 / 温和地</t>
+  </si>
+  <si>
+    <t>位于 / 处于</t>
+  </si>
+  <si>
+    <t>领先的 / 引导的</t>
+  </si>
+  <si>
+    <t>警惕顾虑的</t>
+  </si>
+  <si>
+    <t>锁定 / 锁住</t>
+  </si>
+  <si>
+    <t>观景台 / 展望点</t>
+  </si>
+  <si>
+    <t>秀美郁郁葱葱的</t>
+  </si>
+  <si>
+    <t>匹配 / 符合</t>
+  </si>
+  <si>
+    <t>宏伟强大的</t>
+  </si>
+  <si>
+    <t>留心的 / 注意的</t>
+  </si>
+  <si>
+    <t>新闻 / 消息</t>
+  </si>
+  <si>
+    <t>被遮挡遮蔽的</t>
+  </si>
+  <si>
+    <t>最佳的 / 最理想的</t>
+  </si>
+  <si>
+    <t>井然有序的</t>
+  </si>
+  <si>
+    <t>违约金 / 罚款</t>
+  </si>
+  <si>
+    <t>相关的 / 切题的</t>
+  </si>
+  <si>
+    <t>巅峰 / 顶峰</t>
+  </si>
+  <si>
+    <t>平原 / 简朴的</t>
+  </si>
+  <si>
+    <t>熟练的 / 演练过的</t>
+  </si>
+  <si>
+    <t>赞扬 / 称赞</t>
+  </si>
+  <si>
+    <t>精准 / 精确度</t>
+  </si>
+  <si>
+    <t>蓬松的（云朵）</t>
+  </si>
+  <si>
+    <t>拉 / 吸引</t>
+  </si>
+  <si>
+    <t>排名 / 评级</t>
+  </si>
+  <si>
+    <t>现实 / 实际情况</t>
+  </si>
+  <si>
+    <t>区域 / 地区</t>
+  </si>
+  <si>
+    <t>remaining (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>report (名词/实体)</t>
+  </si>
+  <si>
+    <t>rosemary (名词/实体)</t>
+  </si>
+  <si>
+    <t>ruining (名词/实体)</t>
+  </si>
+  <si>
+    <t>rush (名词/实体)</t>
+  </si>
+  <si>
+    <t>rust (名词/实体)</t>
+  </si>
+  <si>
+    <t>school (名词/实体)</t>
+  </si>
+  <si>
+    <t>secret (名词/实体)</t>
+  </si>
+  <si>
+    <t>securely (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>sensing (名词/实体)</t>
+  </si>
+  <si>
+    <t>severe (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>shining (名词/实体)</t>
+  </si>
+  <si>
+    <t>shortest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>silly (名词/实体)</t>
+  </si>
+  <si>
+    <t>slim (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>snap (名词/实体)</t>
+  </si>
+  <si>
+    <t>snapped (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>sometime (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>squeezed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>stability (名词/实体)</t>
+  </si>
+  <si>
+    <t>staring (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>stick (名词/实体)</t>
+  </si>
+  <si>
+    <t>stormy (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>subject (名词/实体)</t>
+  </si>
+  <si>
+    <t>subtle (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>supporting (名词/实体)</t>
+  </si>
+  <si>
+    <t>surface (名词/实体)</t>
+  </si>
+  <si>
+    <t>tale (名词/实体)</t>
+  </si>
+  <si>
+    <t>talented (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>tentative (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>territory (名词/实体)</t>
+  </si>
+  <si>
+    <t>trained (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>tropical (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>undecided (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>uneven (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unexplainable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unimaginable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unlikely (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>untouched (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>varied (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>warn (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>wasting (名词/实体)</t>
+  </si>
+  <si>
+    <t>abandoned (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>abrupt (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>ache (名词/实体)</t>
+  </si>
+  <si>
+    <t>actively (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>adamant (名词/实体)</t>
+  </si>
+  <si>
+    <t>adept (名词/实体)</t>
+  </si>
+  <si>
+    <t>adequate (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>adjustment (名词/实体)</t>
+  </si>
+  <si>
+    <t>admirably (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>admission (名词/实体)</t>
+  </si>
+  <si>
+    <t>adorable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>adored (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>affect (名词/实体)</t>
+  </si>
+  <si>
+    <t>aggravate (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>aid (名词/实体)</t>
+  </si>
+  <si>
+    <t>airy (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>alike (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>alive (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>altered (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>altering (名词/实体)</t>
+  </si>
+  <si>
+    <t>altogether (名词/实体)</t>
+  </si>
+  <si>
+    <t>amelia (名词/实体)</t>
+  </si>
+  <si>
+    <t>anticipate (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>antsy (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>apocalypse (名词/实体)</t>
+  </si>
+  <si>
+    <t>apology (名词/实体)</t>
+  </si>
+  <si>
+    <t>apparent (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>appease (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>appointed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>appreciative (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>arctic (名词/实体)</t>
+  </si>
+  <si>
+    <t>art (名词/实体)</t>
+  </si>
+  <si>
+    <t>asset (名词/实体)</t>
+  </si>
+  <si>
+    <t>assume (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>assuring (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>atrocious (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>attack (名词/实体)</t>
+  </si>
+  <si>
+    <t>attesting (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>attractive (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>avid (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>avoided (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>avoiding (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>award (名词/实体)</t>
+  </si>
+  <si>
+    <t>babbling (名词/实体)</t>
+  </si>
+  <si>
+    <t>backed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>backing (名词/实体)</t>
+  </si>
+  <si>
+    <t>banner (名词/实体)</t>
+  </si>
+  <si>
+    <t>bearable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>beating (名词/实体)</t>
+  </si>
+  <si>
+    <t>beg (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>belonging (名词/实体)</t>
+  </si>
+  <si>
+    <t>blanket (名词/实体)</t>
+  </si>
+  <si>
+    <t>blasted (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>bless (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>blessing (名词/实体)</t>
+  </si>
+  <si>
+    <t>blindfolded (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>blip (名词/实体)</t>
+  </si>
+  <si>
+    <t>blob (名词/实体)</t>
+  </si>
+  <si>
+    <t>blow (名词/实体)</t>
+  </si>
+  <si>
+    <t>bluff (名词/实体)</t>
+  </si>
+  <si>
+    <t>boiled (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>bolder (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>bond (名词/实体)</t>
+  </si>
+  <si>
+    <t>bottomless (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>bound (名词/实体)</t>
+  </si>
+  <si>
+    <t>brain (名词/实体)</t>
+  </si>
+  <si>
+    <t>brave (名词/实体)</t>
+  </si>
+  <si>
+    <t>breezy (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>brilliantly (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>brown (名词/实体)</t>
+  </si>
+  <si>
+    <t>browse (名词/实体)</t>
+  </si>
+  <si>
+    <t>bug (名词/实体)</t>
+  </si>
+  <si>
+    <t>bumpier (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>bumping (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>buoyant (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>burn (名词/实体)</t>
+  </si>
+  <si>
+    <t>burned (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>burnt (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>bust (名词/实体)</t>
+  </si>
+  <si>
+    <t>buying (名词/实体)</t>
+  </si>
+  <si>
+    <t>buzz (名词/实体)</t>
+  </si>
+  <si>
+    <t>bypass (名词/实体)</t>
+  </si>
+  <si>
+    <t>cast (名词/实体)</t>
+  </si>
+  <si>
+    <t>catty (名词/实体)</t>
+  </si>
+  <si>
+    <t>centerpiece (名词/实体)</t>
+  </si>
+  <si>
+    <t>certified (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>challenge (名词/实体)</t>
+  </si>
+  <si>
+    <t>champ (名词/实体)</t>
+  </si>
+  <si>
+    <t>chaotic (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>character (名词/实体)</t>
+  </si>
+  <si>
+    <t>chargeable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>cheapest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>chicken (名词/实体)</t>
+  </si>
+  <si>
+    <t>chief (名词/实体)</t>
+  </si>
+  <si>
+    <t>chilled (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>cleanest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>cleanliness (名词/实体)</t>
+  </si>
+  <si>
+    <t>clearing (名词/实体)</t>
+  </si>
+  <si>
+    <t>climbed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>closest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>cohesive (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>combine (名词/实体)</t>
+  </si>
+  <si>
+    <t>combining (名词/实体)</t>
+  </si>
+  <si>
+    <t>commercialized (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>committed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>compensate (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>compensated (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>complained (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>completing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>complex (名词/实体)</t>
+  </si>
+  <si>
+    <t>compliance (名词/实体)</t>
+  </si>
+  <si>
+    <t>complimented (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>concerning (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>confused (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>congestion (名词/实体)</t>
+  </si>
+  <si>
+    <t>congratulation (名词/实体)</t>
+  </si>
+  <si>
+    <t>conscience (名词/实体)</t>
+  </si>
+  <si>
+    <t>considerate (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>console (名词/实体)</t>
+  </si>
+  <si>
+    <t>consoling (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>constructive (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>continent (名词/实体)</t>
+  </si>
+  <si>
+    <t>continuous (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>contrary (名词/实体)</t>
+  </si>
+  <si>
+    <t>contributed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>converted (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>coordinate (名词/实体)</t>
+  </si>
+  <si>
+    <t>coordination (名词/实体)</t>
+  </si>
+  <si>
+    <t>cornucopia (名词/实体)</t>
+  </si>
+  <si>
+    <t>corresponding (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>countless (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>coy (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>crane (名词/实体)</t>
+  </si>
+  <si>
+    <t>crappy (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>crazed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>creates (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>criticism (名词/实体)</t>
+  </si>
+  <si>
+    <t>crooked (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>crunch (名词/实体)</t>
+  </si>
+  <si>
+    <t>crusty (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>cry (名词/实体)</t>
+  </si>
+  <si>
+    <t>curt (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>damage (名词/实体)</t>
+  </si>
+  <si>
+    <t>dash (名词/实体)</t>
+  </si>
+  <si>
+    <t>deeper (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>degraded (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>delivering (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>deluxe (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>demonstrated (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>denied (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>denying (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>desirable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>desire (名词/实体)</t>
+  </si>
+  <si>
+    <t>desired (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>dicey (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>dickey (名词/实体)</t>
+  </si>
+  <si>
+    <t>digest (名词/实体)</t>
+  </si>
+  <si>
+    <t>diluted (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>diminish (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>disadvantage (名词/实体)</t>
+  </si>
+  <si>
+    <t>disappear (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>disguise (名词/实体)</t>
+  </si>
+  <si>
+    <t>dislike (名词/实体)</t>
+  </si>
+  <si>
+    <t>dismay (名词/实体)</t>
+  </si>
+  <si>
+    <t>dissipate (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>distortion (名词/实体)</t>
+  </si>
+  <si>
+    <t>district (名词/实体)</t>
+  </si>
+  <si>
+    <t>disturbing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>dos (名词/实体)</t>
+  </si>
+  <si>
+    <t>downfall (名词/实体)</t>
+  </si>
+  <si>
+    <t>downgraded (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>dramatically (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>dreaming (名词/实体)</t>
+  </si>
+  <si>
+    <t>dressed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>dubbed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>dud (名词/实体)</t>
+  </si>
+  <si>
+    <t>duke (名词/实体)</t>
+  </si>
+  <si>
+    <t>dumb (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>dynamic (名词/实体)</t>
+  </si>
+  <si>
+    <t>echo (名词/实体)</t>
+  </si>
+  <si>
+    <t>eden (名词/实体)</t>
+  </si>
+  <si>
+    <t>educate (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>element (名词/实体)</t>
+  </si>
+  <si>
+    <t>elusive (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>enables (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>enabling (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>encompassing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>encouragement (名词/实体)</t>
+  </si>
+  <si>
+    <t>endeavor (名词/实体)</t>
+  </si>
+  <si>
+    <t>endless (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>endorse (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>endure (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>enhance (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>enlightening (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>ethical (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>everlasting (名词/实体)</t>
+  </si>
+  <si>
+    <t>excellently (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>excuse (名词/实体)</t>
+  </si>
+  <si>
+    <t>exhausting (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>existent (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>exposure (名词/实体)</t>
+  </si>
+  <si>
+    <t>extends (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>extolled (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>fab (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>facing (名词/实体)</t>
+  </si>
+  <si>
+    <t>fail (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>failing (名词/实体)</t>
+  </si>
+  <si>
+    <t>faint (名词/实体)</t>
+  </si>
+  <si>
+    <t>false (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>familiarity (名词/实体)</t>
+  </si>
+  <si>
+    <t>fantasy (名词/实体)</t>
+  </si>
+  <si>
+    <t>fat (名词/实体)</t>
+  </si>
+  <si>
+    <t>fatality (名词/实体)</t>
+  </si>
+  <si>
+    <t>faulty (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>favor (名词/实体)</t>
+  </si>
+  <si>
+    <t>favorable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>feared (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>feat (名词/实体)</t>
+  </si>
+  <si>
+    <t>featured (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>feed (名词/实体)</t>
+  </si>
+  <si>
+    <t>final (名词/实体)</t>
+  </si>
+  <si>
+    <t>fired (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>firm (名词/实体)</t>
+  </si>
+  <si>
+    <t>flash (名词/实体)</t>
+  </si>
+  <si>
+    <t>flood (名词/实体)</t>
+  </si>
+  <si>
+    <t>flooded (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>flop (名词/实体)</t>
+  </si>
+  <si>
+    <t>focussed (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>fond (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>ford (名词/实体)</t>
+  </si>
+  <si>
+    <t>foremost (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>forgetting (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>forgo (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>formal (名词/实体)</t>
+  </si>
+  <si>
+    <t>formidable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>forthright (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>frankly (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>freak (名词/实体)</t>
+  </si>
+  <si>
+    <t>freaked (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>freaking (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>friendliest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>frowning (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>fulfillment (名词/实体)</t>
+  </si>
+  <si>
+    <t>funky (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>gained (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>gca (名词/实体)</t>
+  </si>
+  <si>
+    <t>generic (名词/实体)</t>
+  </si>
+  <si>
+    <t>gimmick (名词/实体)</t>
+  </si>
+  <si>
+    <t>glaciated (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>gloom (名词/实体)</t>
+  </si>
+  <si>
+    <t>glow (名词/实体)</t>
+  </si>
+  <si>
+    <t>goodness (名词/实体)</t>
+  </si>
+  <si>
+    <t>gourmet (名词/实体)</t>
+  </si>
+  <si>
+    <t>graphic (名词/实体)</t>
+  </si>
+  <si>
+    <t>greener (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>grip (名词/实体)</t>
+  </si>
+  <si>
+    <t>gripe (名词/实体)</t>
+  </si>
+  <si>
+    <t>grouping (名词/实体)</t>
+  </si>
+  <si>
+    <t>gruffness (名词/实体)</t>
+  </si>
+  <si>
+    <t>guaranteeing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>gushing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>hairless (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>ham (名词/实体)</t>
+  </si>
+  <si>
+    <t>handicap (名词/实体)</t>
+  </si>
+  <si>
+    <t>handicraft (名词/实体)</t>
+  </si>
+  <si>
+    <t>hardest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>harried (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>health (名词/实体)</t>
+  </si>
+  <si>
+    <t>heap (名词/实体)</t>
+  </si>
+  <si>
+    <t>heating (名词/实体)</t>
+  </si>
+  <si>
+    <t>heavier (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>heaviest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>heavily (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>hero (名词/实体)</t>
+  </si>
+  <si>
+    <t>hesitancy (名词/实体)</t>
+  </si>
+  <si>
+    <t>hint (名词/实体)</t>
+  </si>
+  <si>
+    <t>hitting (名词/实体)</t>
+  </si>
+  <si>
+    <t>hole (名词/实体)</t>
+  </si>
+  <si>
+    <t>homey (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>horribly (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>humble (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>humoured (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>husky (名词/实体)</t>
+  </si>
+  <si>
+    <t>hygiene (名词/实体)</t>
+  </si>
+  <si>
+    <t>illustrate (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>inclined (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>incomparable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>independently (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>induced (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>indulged (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>industrial (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>inquired (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>inspire (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>inspires (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>instructing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>interfering (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>intolerable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>invasive (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>itching (名词/实体)</t>
+  </si>
+  <si>
+    <t>jackpot (名词/实体)</t>
+  </si>
+  <si>
+    <t>jarring (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>jerky (名词/实体)</t>
+  </si>
+  <si>
+    <t>joked (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>kill (名词/实体)</t>
+  </si>
+  <si>
+    <t>kindest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>knock (名词/实体)</t>
+  </si>
+  <si>
+    <t>kudos (名词/实体)</t>
+  </si>
+  <si>
+    <t>labeled (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>lapse (名词/实体)</t>
+  </si>
+  <si>
+    <t>largest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>lean (名词/实体)</t>
+  </si>
+  <si>
+    <t>lecture (名词/实体)</t>
+  </si>
+  <si>
+    <t>legitimacy (名词/实体)</t>
+  </si>
+  <si>
+    <t>leisured (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>lends (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>lenient (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>leper (名词/实体)</t>
+  </si>
+  <si>
+    <t>limitation (名词/实体)</t>
+  </si>
+  <si>
+    <t>limitless (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>lined (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>lively (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>locking (名词/实体)</t>
+  </si>
+  <si>
+    <t>loose (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>lose (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>loss (名词/实体)</t>
+  </si>
+  <si>
+    <t>lover (名词/实体)</t>
+  </si>
+  <si>
+    <t>lowered (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>magnificently (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>mar (名词/实体)</t>
+  </si>
+  <si>
+    <t>marriage (名词/实体)</t>
+  </si>
+  <si>
+    <t>master (名词/实体)</t>
+  </si>
+  <si>
+    <t>material (名词/实体)</t>
+  </si>
+  <si>
+    <t>meaningful (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>measure (名词/实体)</t>
+  </si>
+  <si>
+    <t>melted (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>merry (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>mess (名词/实体)</t>
+  </si>
+  <si>
+    <t>method (名词/实体)</t>
+  </si>
+  <si>
+    <t>minimising (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>minimizing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>minus (名词/实体)</t>
+  </si>
+  <si>
+    <t>miracle (名词/实体)</t>
+  </si>
+  <si>
+    <t>mitigate (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>modernized (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>modified (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>motorway (名词/实体)</t>
+  </si>
+  <si>
+    <t>mule (名词/实体)</t>
+  </si>
+  <si>
+    <t>musical (名词/实体)</t>
+  </si>
+  <si>
+    <t>mystical (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>neck (名词/实体)</t>
+  </si>
+  <si>
+    <t>nerd (名词/实体)</t>
+  </si>
+  <si>
+    <t>nestled (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>nimble (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>nonetheless (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>nose (名词/实体)</t>
+  </si>
+  <si>
+    <t>nostalgic (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>noted (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>obliged (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>obnoxious (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>occur (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>occurred (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>oddly (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>outright (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>oversized (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>paraplegic (名词/实体)</t>
+  </si>
+  <si>
+    <t>passable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>passport (名词/实体)</t>
+  </si>
+  <si>
+    <t>perception (名词/实体)</t>
+  </si>
+  <si>
+    <t>perfection (名词/实体)</t>
+  </si>
+  <si>
+    <t>pest (名词/实体)</t>
+  </si>
+  <si>
+    <t>pierce (名词/实体)</t>
+  </si>
+  <si>
+    <t>pit (名词/实体)</t>
+  </si>
+  <si>
+    <t>plastic (名词/实体)</t>
+  </si>
+  <si>
+    <t>playful (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>pleasantness (名词/实体)</t>
+  </si>
+  <si>
+    <t>poetic (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>polish (名词/实体)</t>
+  </si>
+  <si>
+    <t>pound (名词/实体)</t>
+  </si>
+  <si>
+    <t>practical (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>practice (名词/实体)</t>
+  </si>
+  <si>
+    <t>precisely (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>preference (名词/实体)</t>
+  </si>
+  <si>
+    <t>pregnant (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>premium (名词/实体)</t>
+  </si>
+  <si>
+    <t>presence (名词/实体)</t>
+  </si>
+  <si>
+    <t>preserve (名词/实体)</t>
+  </si>
+  <si>
+    <t>pricier (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>prime (名词/实体)</t>
+  </si>
+  <si>
+    <t>probability (名词/实体)</t>
+  </si>
+  <si>
+    <t>prominent (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>propensity (名词/实体)</t>
+  </si>
+  <si>
+    <t>prospect (名词/实体)</t>
+  </si>
+  <si>
+    <t>purple (名词/实体)</t>
+  </si>
+  <si>
+    <t>push (名词/实体)</t>
+  </si>
+  <si>
+    <t>pushed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>questioned (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>rail (名词/实体)</t>
+  </si>
+  <si>
+    <t>raising (名词/实体)</t>
+  </si>
+  <si>
+    <t>rally (名词/实体)</t>
+  </si>
+  <si>
+    <t>ranking (名词/实体)</t>
+  </si>
+  <si>
+    <t>rapid (名词/实体)</t>
+  </si>
+  <si>
+    <t>raw (名词/实体)</t>
+  </si>
+  <si>
+    <t>readily (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>realised (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>recall (名词/实体)</t>
+  </si>
+  <si>
+    <t>receives (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>receiving (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>recovery (名词/实体)</t>
+  </si>
+  <si>
+    <t>reflecting (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>reflects (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>refusing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>regent (名词/实体)</t>
+  </si>
+  <si>
+    <t>relative (名词/实体)</t>
+  </si>
+  <si>
+    <t>remark (名词/实体)</t>
+  </si>
+  <si>
+    <t>removed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>removing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>rendering (名词/实体)</t>
+  </si>
+  <si>
+    <t>replaced (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>reported (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>reporting (名词/实体)</t>
+  </si>
+  <si>
+    <t>represent (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>represents (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>rescue (名词/实体)</t>
+  </si>
+  <si>
+    <t>resounding (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>responsibility (名词/实体)</t>
+  </si>
+  <si>
+    <t>restraint (名词/实体)</t>
+  </si>
+  <si>
+    <t>retiring (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>revived (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>revolting (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>reward (名词/实体)</t>
+  </si>
+  <si>
+    <t>richer (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>rig (名词/实体)</t>
+  </si>
+  <si>
+    <t>rigorous (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>rising (名词/实体)</t>
+  </si>
+  <si>
+    <t>risking (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>risky (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>roaring (名词/实体)</t>
+  </si>
+  <si>
+    <t>rose (名词/实体)</t>
+  </si>
+  <si>
+    <t>royal (名词/实体)</t>
+  </si>
+  <si>
+    <t>rued (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>ruffling (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>ruin (名词/实体)</t>
+  </si>
+  <si>
+    <t>rusty (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>sacred (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>sainthood (名词/实体)</t>
+  </si>
+  <si>
+    <t>salt (名词/实体)</t>
+  </si>
+  <si>
+    <t>salvaging (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>satisfaction (名词/实体)</t>
+  </si>
+  <si>
+    <t>satisfactorily (程度/方式副词)</t>
+  </si>
+  <si>
+    <t>satisfactory (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>seal (名词/实体)</t>
+  </si>
+  <si>
+    <t>sealed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>seemless (客观/中性/过程词)</t>
+  </si>
+  <si>
+    <t>separated (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>serve (名词/实体)</t>
+  </si>
+  <si>
+    <t>sexy (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>shadow (名词/实体)</t>
+  </si>
+  <si>
+    <t>shifted (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>shiny (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>shipwreck (名词/实体)</t>
+  </si>
+  <si>
+    <t>shoot (名词/实体)</t>
+  </si>
+  <si>
+    <t>signature (名词/实体)</t>
+  </si>
+  <si>
+    <t>sincere (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>sits (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>smarter (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>smelled (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>smelling (名词/实体)</t>
+  </si>
+  <si>
+    <t>snafu (名词/实体)</t>
+  </si>
+  <si>
+    <t>snowed (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>soften (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>soil (名词/实体)</t>
+  </si>
+  <si>
+    <t>specialized (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>spoiling (名词/实体)</t>
+  </si>
+  <si>
+    <t>sport (名词/实体)</t>
+  </si>
+  <si>
+    <t>spouting (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>statement (名词/实体)</t>
+  </si>
+  <si>
+    <t>steam (名词/实体)</t>
+  </si>
+  <si>
+    <t>steep (名词/实体)</t>
+  </si>
+  <si>
+    <t>sticking (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>stiller (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>stillness (名词/实体)</t>
+  </si>
+  <si>
+    <t>sting (名词/实体)</t>
+  </si>
+  <si>
+    <t>stinky (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>straightforward (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>stranger (名词/实体)</t>
+  </si>
+  <si>
+    <t>strength (名词/实体)</t>
+  </si>
+  <si>
+    <t>strenuous (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>stronger (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>substitute (名词/实体)</t>
+  </si>
+  <si>
+    <t>success (名词/实体)</t>
+  </si>
+  <si>
+    <t>suck (名词/实体)</t>
+  </si>
+  <si>
+    <t>suffers (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>sufficient (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>suited (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>sunshine (名词/实体)</t>
+  </si>
+  <si>
+    <t>surprising (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>suspected (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>swallow (名词/实体)</t>
+  </si>
+  <si>
+    <t>swamp (名词/实体)</t>
+  </si>
+  <si>
+    <t>swan (名词/实体)</t>
+  </si>
+  <si>
+    <t>swear (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>sweeter (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>sweetheart (名词/实体)</t>
+  </si>
+  <si>
+    <t>swell (名词/实体)</t>
+  </si>
+  <si>
+    <t>swinging (名词/实体)</t>
+  </si>
+  <si>
+    <t>sympathetic (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>tactile (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>taller (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>teach (名词/实体)</t>
+  </si>
+  <si>
+    <t>teary (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>tendency (名词/实体)</t>
+  </si>
+  <si>
+    <t>tender (名词/实体)</t>
+  </si>
+  <si>
+    <t>tends (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>test (名词/实体)</t>
+  </si>
+  <si>
+    <t>thickest (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>thirsty (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>throwing (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>timeless (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>topper (名词/实体)</t>
+  </si>
+  <si>
+    <t>topping (名词/实体)</t>
+  </si>
+  <si>
+    <t>totality (名词/实体)</t>
+  </si>
+  <si>
+    <t>tragic (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>transparency (名词/实体)</t>
+  </si>
+  <si>
+    <t>trek (名词/实体)</t>
+  </si>
+  <si>
+    <t>trick (名词/实体)</t>
+  </si>
+  <si>
+    <t>tropic (名词/实体)</t>
+  </si>
+  <si>
+    <t>uncharted (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>understated (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>unethical (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unhelpful (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unimpressed (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>uninhabited (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>uninterested (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unloaded (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>unlucky (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unpaved (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unrivalled (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unsurpassable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>unusual (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>upbeat (名词/实体)</t>
+  </si>
+  <si>
+    <t>vain (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>valued (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>vanish (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>vary (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>varying (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>verify (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>vernal (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>versed (名词/实体)</t>
+  </si>
+  <si>
+    <t>viable (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>victory (名词/实体)</t>
+  </si>
+  <si>
+    <t>waived (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>wander (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>wandered (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>warmer (名词/实体)</t>
+  </si>
+  <si>
+    <t>watchful (中性/客观属性形容词)</t>
+  </si>
+  <si>
+    <t>weary (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>weathered (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>weep (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>wisdom (名词/实体)</t>
+  </si>
+  <si>
+    <t>woke (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>yearly (名词/实体)</t>
+  </si>
+  <si>
+    <t>yelling (名词/实体)</t>
+  </si>
+  <si>
+    <t>yielded (过程/动作动词)</t>
+  </si>
+  <si>
+    <t>youngest (中性/客观属性形容词)</t>
   </si>
   <si>
     <t>review_a621d61d85c6d1941fd94167 :: Our Misty Fjords tour was a boat ride from Ketchican to the fjords, with a return by small plane.  The guides on the boat were informative and nice.  

</xml_diff>